<commit_message>
EXP_V121 | 10/04/25 | 23:23
</commit_message>
<xml_diff>
--- a/03_BOM/EXP_V121_BOM.xlsx
+++ b/03_BOM/EXP_V121_BOM.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\LAB\NANORACK_V2_EXP_1.1.1_HW\03_BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77A7ECBC-469D-4FC7-8BC2-1A2654D95408}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A937BEFA-7226-409A-AC31-ECC371012012}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{7FE79776-13CA-40B3-9449-222C1E26C344}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{CB84624A-87DC-4816-B95B-F0221E4A3080}"/>
   </bookViews>
   <sheets>
-    <sheet name="EXP_V121_BOM" sheetId="1" r:id="rId1"/>
+    <sheet name="EXP_V121_BOM1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Titles" localSheetId="0">EXP_V121_BOM!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">EXP_V121_BOM1!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="405" uniqueCount="297">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="405" uniqueCount="298">
   <si>
     <t>Name</t>
   </si>
@@ -489,7 +489,7 @@
     <t>22R</t>
   </si>
   <si>
-    <t>R4, R8, R15, R25, R26, R45, R47, R48, R49, R50, R51, R52, R53, R54, R55, R66, R67, R68, R69, R72, R73, R74, R75, R78, R79, R80, R81, R84, R85, R86, R87, R94, R95, R96, R97, R105, R106, R107, R113, R114, R115, R116, R117, R118, R119, R120, R121, R122, R123, R124, R125, R126, R127, R128, R129, R130, R131, R132, R133, R134, R141, R142, R143, R144, R154, R157, R159, R161, R162</t>
+    <t>R4, R8, R15, R25, R26, R45, R47, R48, R49, R50, R51, R52, R53, R54, R55, R66, R67, R68, R69, R72, R73, R74, R75, R78, R79, R80, R81, R84, R85, R86, R87, R94, R95, R96, R97, R105, R106, R107, R113, R114, R115, R116, R117, R118, R119, R120, R121, R122, R123, R124, R125, R126, R127, R128, R129, R130, R131, R132, R133, R134, R141, R142, R143, R144, R154, R157, R159, R161, R162, R167</t>
   </si>
   <si>
     <t>ERJ-3EKF22R0V</t>
@@ -696,7 +696,7 @@
     <t>U9</t>
   </si>
   <si>
-    <t>ADM3065EARZ</t>
+    <t>MAX3485EESA+</t>
   </si>
   <si>
     <t>IC TRANSCEIVER HALF 1/1 8SOIC</t>
@@ -706,6 +706,9 @@
   </si>
   <si>
     <t>SOIC8_3.9mm</t>
+  </si>
+  <si>
+    <t>Maxim</t>
   </si>
   <si>
     <t>MCP4921-E/SN</t>
@@ -1294,17 +1297,17 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{23992843-3C56-4E9C-9DDF-BB2CA52796F1}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{81B74A45-8FA9-438A-BE1B-5C4E575BDB90}">
   <dimension ref="A1:G69"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.7109375" customWidth="1"/>
-    <col min="2" max="2" width="65.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="72.42578125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="32" customWidth="1"/>
     <col min="4" max="4" width="10.85546875" customWidth="1"/>
-    <col min="5" max="5" width="47.7109375" customWidth="1"/>
+    <col min="5" max="5" width="36.28515625" customWidth="1"/>
     <col min="6" max="6" width="16.42578125" customWidth="1"/>
-    <col min="7" max="7" width="27" customWidth="1"/>
+    <col min="7" max="7" width="31.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -1358,7 +1361,7 @@
         <v>13</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>14</v>
@@ -1381,7 +1384,7 @@
         <v>18</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>20</v>
@@ -1404,7 +1407,7 @@
         <v>24</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>25</v>
@@ -1427,7 +1430,7 @@
         <v>27</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>28</v>
@@ -1450,7 +1453,7 @@
         <v>30</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>31</v>
@@ -1473,7 +1476,7 @@
         <v>32</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>33</v>
@@ -1496,7 +1499,7 @@
         <v>35</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>36</v>
@@ -1519,7 +1522,7 @@
         <v>38</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>39</v>
@@ -1542,7 +1545,7 @@
         <v>41</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>42</v>
@@ -1565,7 +1568,7 @@
         <v>45</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>46</v>
@@ -1588,7 +1591,7 @@
         <v>48</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>49</v>
@@ -1657,7 +1660,7 @@
         <v>61</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>62</v>
@@ -1680,7 +1683,7 @@
         <v>66</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="C17" s="2" t="s">
         <v>67</v>
@@ -1703,7 +1706,7 @@
         <v>69</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C18" s="2" t="s">
         <v>70</v>
@@ -1726,7 +1729,7 @@
         <v>72</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="C19" s="2" t="s">
         <v>73</v>
@@ -1791,7 +1794,7 @@
         <v>82</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="C22" s="2" t="s">
         <v>83</v>
@@ -2028,7 +2031,7 @@
         <v>123</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C33" s="2" t="s">
         <v>124</v>
@@ -2074,7 +2077,7 @@
         <v>131</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="C35" s="2" t="s">
         <v>132</v>
@@ -2120,7 +2123,7 @@
         <v>141</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="C37" s="2" t="s">
         <v>142</v>
@@ -2143,7 +2146,7 @@
         <v>146</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="C38" s="2" t="s">
         <v>147</v>
@@ -2166,7 +2169,7 @@
         <v>149</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="C39" s="2" t="s">
         <v>150</v>
@@ -2189,13 +2192,13 @@
         <v>152</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="C40" s="2" t="s">
         <v>153</v>
       </c>
       <c r="D40" s="1">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E40" s="2" t="s">
         <v>143</v>
@@ -2212,7 +2215,7 @@
         <v>155</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="C41" s="2" t="s">
         <v>156</v>
@@ -2235,7 +2238,7 @@
         <v>158</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C42" s="2" t="s">
         <v>159</v>
@@ -2258,7 +2261,7 @@
         <v>161</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="C43" s="2" t="s">
         <v>162</v>
@@ -2281,7 +2284,7 @@
         <v>164</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C44" s="2" t="s">
         <v>165</v>
@@ -2304,7 +2307,7 @@
         <v>167</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="C45" s="2" t="s">
         <v>168</v>
@@ -2327,7 +2330,7 @@
         <v>170</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="C46" s="2" t="s">
         <v>171</v>
@@ -2350,7 +2353,7 @@
         <v>173</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C47" s="2" t="s">
         <v>174</v>
@@ -2373,7 +2376,7 @@
         <v>176</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="C48" s="2" t="s">
         <v>177</v>
@@ -2396,7 +2399,7 @@
         <v>179</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="C49" s="2" t="s">
         <v>180</v>
@@ -2419,7 +2422,7 @@
         <v>182</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="C50" s="2" t="s">
         <v>183</v>
@@ -2442,7 +2445,7 @@
         <v>185</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="C51" s="2" t="s">
         <v>186</v>
@@ -2465,7 +2468,7 @@
         <v>188</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="C52" s="2" t="s">
         <v>189</v>
@@ -2511,7 +2514,7 @@
         <v>196</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="C54" s="2" t="s">
         <v>197</v>
@@ -2557,7 +2560,7 @@
         <v>204</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="C56" s="2" t="s">
         <v>205</v>
@@ -2684,7 +2687,7 @@
         <v>225</v>
       </c>
       <c r="F61" s="2" t="s">
-        <v>217</v>
+        <v>226</v>
       </c>
       <c r="G61" s="2" t="s">
         <v>222</v>
@@ -2692,186 +2695,186 @@
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="2" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="D62" s="1">
         <v>4</v>
       </c>
       <c r="E62" s="2" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="F62" s="2" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="G62" s="2" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="C63" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="D63" s="1">
+        <v>1</v>
+      </c>
+      <c r="E63" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="F63" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="G63" s="2" t="s">
         <v>232</v>
-      </c>
-      <c r="D63" s="1">
-        <v>1</v>
-      </c>
-      <c r="E63" s="2" t="s">
-        <v>233</v>
-      </c>
-      <c r="F63" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="G63" s="2" t="s">
-        <v>231</v>
       </c>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="2" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="D64" s="1">
         <v>4</v>
       </c>
       <c r="E64" s="2" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="F64" s="2" t="s">
         <v>203</v>
       </c>
       <c r="G64" s="2" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A65" s="2" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="D65" s="1">
         <v>2</v>
       </c>
       <c r="E65" s="2" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="F65" s="2" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="G65" s="2" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="B66" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="C66" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="D66" s="1">
+        <v>1</v>
+      </c>
+      <c r="E66" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="F66" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="G66" s="2" t="s">
         <v>243</v>
-      </c>
-      <c r="C66" s="2" t="s">
-        <v>244</v>
-      </c>
-      <c r="D66" s="1">
-        <v>1</v>
-      </c>
-      <c r="E66" s="2" t="s">
-        <v>245</v>
-      </c>
-      <c r="F66" s="2" t="s">
-        <v>246</v>
-      </c>
-      <c r="G66" s="2" t="s">
-        <v>242</v>
       </c>
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A67" s="2" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="B67" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="C67" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="D67" s="1">
+        <v>1</v>
+      </c>
+      <c r="E67" s="2" t="s">
         <v>248</v>
-      </c>
-      <c r="C67" s="2" t="s">
-        <v>249</v>
-      </c>
-      <c r="D67" s="1">
-        <v>1</v>
-      </c>
-      <c r="E67" s="2" t="s">
-        <v>247</v>
       </c>
       <c r="F67" s="2" t="s">
         <v>203</v>
       </c>
       <c r="G67" s="2" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="B68" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="C68" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="D68" s="1">
+        <v>1</v>
+      </c>
+      <c r="E68" s="2" t="s">
         <v>251</v>
       </c>
-      <c r="C68" s="2" t="s">
-        <v>252</v>
-      </c>
-      <c r="D68" s="1">
-        <v>1</v>
-      </c>
-      <c r="E68" s="2" t="s">
-        <v>250</v>
-      </c>
       <c r="F68" s="2" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="G68" s="2" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A69" s="2" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="D69" s="1">
         <v>1</v>
       </c>
       <c r="E69" s="2" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="F69" s="2" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="G69" s="2" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
EXP_V121 | 11/04/25 | 14:17
</commit_message>
<xml_diff>
--- a/03_BOM/EXP_V121_BOM.xlsx
+++ b/03_BOM/EXP_V121_BOM.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\LAB\NANORACK_V2_EXP_1.1.1_HW\03_BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A937BEFA-7226-409A-AC31-ECC371012012}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2F194ED-F795-427F-8A37-495763D98C9D}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{CB84624A-87DC-4816-B95B-F0221E4A3080}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{CB84624A-87DC-4816-B95B-F0221E4A3080}"/>
   </bookViews>
   <sheets>
     <sheet name="EXP_V121_BOM1" sheetId="1" r:id="rId1"/>
@@ -498,9 +498,6 @@
     <t>4.7k</t>
   </si>
   <si>
-    <t>R5, R40, R41, R42, R43, R44, R90, R91, R92, R93, R99, R100, R139, R140, R153, R155, R163, R164, R165, R166</t>
-  </si>
-  <si>
     <t>ERJ-3EKF4701V</t>
   </si>
   <si>
@@ -922,6 +919,9 @@
   </si>
   <si>
     <t>IC REDRIVER I2C HOTSWAP 8TSSOP</t>
+  </si>
+  <si>
+    <t>R5, R40, R41, R42, R43, R44, R90, R91, R92, R93, R99, R100, R139, R140, R153, R155, R163, R164, R165, R166, R168</t>
   </si>
 </sst>
 </file>
@@ -1299,18 +1299,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{81B74A45-8FA9-438A-BE1B-5C4E575BDB90}">
   <dimension ref="A1:G69"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.7109375" customWidth="1"/>
-    <col min="2" max="2" width="72.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.7265625" customWidth="1"/>
+    <col min="2" max="2" width="72.453125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="32" customWidth="1"/>
-    <col min="4" max="4" width="10.85546875" customWidth="1"/>
-    <col min="5" max="5" width="36.28515625" customWidth="1"/>
-    <col min="6" max="6" width="16.42578125" customWidth="1"/>
-    <col min="7" max="7" width="31.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.81640625" customWidth="1"/>
+    <col min="5" max="5" width="36.26953125" customWidth="1"/>
+    <col min="6" max="6" width="16.453125" customWidth="1"/>
+    <col min="7" max="7" width="31.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -1333,7 +1333,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>7</v>
       </c>
@@ -1356,12 +1356,12 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>13</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>14</v>
@@ -1379,12 +1379,12 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>18</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>20</v>
@@ -1402,12 +1402,12 @@
         <v>23</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>24</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>25</v>
@@ -1425,12 +1425,12 @@
         <v>26</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>27</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>28</v>
@@ -1448,12 +1448,12 @@
         <v>29</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>30</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>31</v>
@@ -1471,12 +1471,12 @@
         <v>29</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>32</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>33</v>
@@ -1494,12 +1494,12 @@
         <v>34</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
         <v>35</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>36</v>
@@ -1517,12 +1517,12 @@
         <v>37</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>38</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>39</v>
@@ -1540,12 +1540,12 @@
         <v>40</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>41</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>42</v>
@@ -1563,12 +1563,12 @@
         <v>44</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>45</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>46</v>
@@ -1586,12 +1586,12 @@
         <v>47</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>48</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>49</v>
@@ -1609,7 +1609,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>51</v>
       </c>
@@ -1632,7 +1632,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>56</v>
       </c>
@@ -1655,12 +1655,12 @@
         <v>56</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
         <v>61</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>62</v>
@@ -1678,12 +1678,12 @@
         <v>65</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
         <v>66</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="C17" s="2" t="s">
         <v>67</v>
@@ -1701,12 +1701,12 @@
         <v>68</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
         <v>69</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="C18" s="2" t="s">
         <v>70</v>
@@ -1724,12 +1724,12 @@
         <v>71</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
         <v>72</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="C19" s="2" t="s">
         <v>73</v>
@@ -1747,7 +1747,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
         <v>75</v>
       </c>
@@ -1766,7 +1766,7 @@
       <c r="F20" s="1"/>
       <c r="G20" s="1"/>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A21" s="2" t="s">
         <v>78</v>
       </c>
@@ -1789,12 +1789,12 @@
         <v>78</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A22" s="2" t="s">
         <v>82</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="C22" s="2" t="s">
         <v>83</v>
@@ -1812,7 +1812,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A23" s="2" t="s">
         <v>86</v>
       </c>
@@ -1835,7 +1835,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A24" s="2" t="s">
         <v>90</v>
       </c>
@@ -1858,7 +1858,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A25" s="2" t="s">
         <v>93</v>
       </c>
@@ -1877,7 +1877,7 @@
       <c r="F25" s="1"/>
       <c r="G25" s="1"/>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A26" s="2" t="s">
         <v>97</v>
       </c>
@@ -1900,7 +1900,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A27" s="2" t="s">
         <v>102</v>
       </c>
@@ -1923,7 +1923,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
         <v>106</v>
       </c>
@@ -1942,7 +1942,7 @@
       <c r="F28" s="1"/>
       <c r="G28" s="1"/>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A29" s="2" t="s">
         <v>109</v>
       </c>
@@ -1965,7 +1965,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A30" s="2" t="s">
         <v>114</v>
       </c>
@@ -1984,7 +1984,7 @@
       <c r="F30" s="1"/>
       <c r="G30" s="1"/>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A31" s="2" t="s">
         <v>114</v>
       </c>
@@ -2003,7 +2003,7 @@
       <c r="F31" s="1"/>
       <c r="G31" s="1"/>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A32" s="2" t="s">
         <v>118</v>
       </c>
@@ -2026,12 +2026,12 @@
         <v>118</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A33" s="2" t="s">
         <v>123</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="C33" s="2" t="s">
         <v>124</v>
@@ -2049,7 +2049,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A34" s="2" t="s">
         <v>127</v>
       </c>
@@ -2072,12 +2072,12 @@
         <v>128</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A35" s="2" t="s">
         <v>131</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="C35" s="2" t="s">
         <v>132</v>
@@ -2095,7 +2095,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A36" s="2" t="s">
         <v>136</v>
       </c>
@@ -2118,12 +2118,12 @@
         <v>136</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A37" s="2" t="s">
         <v>141</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="C37" s="2" t="s">
         <v>142</v>
@@ -2141,12 +2141,12 @@
         <v>145</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A38" s="2" t="s">
         <v>146</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="C38" s="2" t="s">
         <v>147</v>
@@ -2164,12 +2164,12 @@
         <v>148</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A39" s="2" t="s">
         <v>149</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="C39" s="2" t="s">
         <v>150</v>
@@ -2187,12 +2187,12 @@
         <v>151</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A40" s="2" t="s">
         <v>152</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="C40" s="2" t="s">
         <v>153</v>
@@ -2210,18 +2210,18 @@
         <v>154</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A41" s="2" t="s">
         <v>155</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>156</v>
+        <v>297</v>
       </c>
       <c r="D41" s="1">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E41" s="2" t="s">
         <v>143</v>
@@ -2230,18 +2230,18 @@
         <v>144</v>
       </c>
       <c r="G41" s="2" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A42" s="2" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A42" s="2" t="s">
+      <c r="B42" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="C42" s="2" t="s">
         <v>158</v>
-      </c>
-      <c r="B42" s="2" t="s">
-        <v>283</v>
-      </c>
-      <c r="C42" s="2" t="s">
-        <v>159</v>
       </c>
       <c r="D42" s="1">
         <v>1</v>
@@ -2253,18 +2253,18 @@
         <v>144</v>
       </c>
       <c r="G42" s="2" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A43" s="2" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A43" s="2" t="s">
+      <c r="B43" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="C43" s="2" t="s">
         <v>161</v>
-      </c>
-      <c r="B43" s="2" t="s">
-        <v>284</v>
-      </c>
-      <c r="C43" s="2" t="s">
-        <v>162</v>
       </c>
       <c r="D43" s="1">
         <v>9</v>
@@ -2276,18 +2276,18 @@
         <v>144</v>
       </c>
       <c r="G43" s="2" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A44" s="2" t="s">
         <v>163</v>
       </c>
-    </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A44" s="2" t="s">
+      <c r="B44" s="2" t="s">
+        <v>284</v>
+      </c>
+      <c r="C44" s="2" t="s">
         <v>164</v>
-      </c>
-      <c r="B44" s="2" t="s">
-        <v>285</v>
-      </c>
-      <c r="C44" s="2" t="s">
-        <v>165</v>
       </c>
       <c r="D44" s="1">
         <v>5</v>
@@ -2299,18 +2299,18 @@
         <v>144</v>
       </c>
       <c r="G44" s="2" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A45" s="2" t="s">
         <v>166</v>
       </c>
-    </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A45" s="2" t="s">
+      <c r="B45" s="2" t="s">
+        <v>285</v>
+      </c>
+      <c r="C45" s="2" t="s">
         <v>167</v>
-      </c>
-      <c r="B45" s="2" t="s">
-        <v>286</v>
-      </c>
-      <c r="C45" s="2" t="s">
-        <v>168</v>
       </c>
       <c r="D45" s="1">
         <v>1</v>
@@ -2322,18 +2322,18 @@
         <v>144</v>
       </c>
       <c r="G45" s="2" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A46" s="2" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A46" s="2" t="s">
+      <c r="B46" s="2" t="s">
+        <v>286</v>
+      </c>
+      <c r="C46" s="2" t="s">
         <v>170</v>
-      </c>
-      <c r="B46" s="2" t="s">
-        <v>287</v>
-      </c>
-      <c r="C46" s="2" t="s">
-        <v>171</v>
       </c>
       <c r="D46" s="1">
         <v>6</v>
@@ -2345,18 +2345,18 @@
         <v>144</v>
       </c>
       <c r="G46" s="2" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A47" s="2" t="s">
         <v>172</v>
       </c>
-    </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A47" s="2" t="s">
+      <c r="B47" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="C47" s="2" t="s">
         <v>173</v>
-      </c>
-      <c r="B47" s="2" t="s">
-        <v>288</v>
-      </c>
-      <c r="C47" s="2" t="s">
-        <v>174</v>
       </c>
       <c r="D47" s="1">
         <v>1</v>
@@ -2368,18 +2368,18 @@
         <v>144</v>
       </c>
       <c r="G47" s="2" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A48" s="2" t="s">
         <v>175</v>
       </c>
-    </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A48" s="2" t="s">
+      <c r="B48" s="2" t="s">
+        <v>288</v>
+      </c>
+      <c r="C48" s="2" t="s">
         <v>176</v>
-      </c>
-      <c r="B48" s="2" t="s">
-        <v>289</v>
-      </c>
-      <c r="C48" s="2" t="s">
-        <v>177</v>
       </c>
       <c r="D48" s="1">
         <v>4</v>
@@ -2391,18 +2391,18 @@
         <v>144</v>
       </c>
       <c r="G48" s="2" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A49" s="2" t="s">
         <v>178</v>
       </c>
-    </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A49" s="2" t="s">
+      <c r="B49" s="2" t="s">
+        <v>289</v>
+      </c>
+      <c r="C49" s="2" t="s">
         <v>179</v>
-      </c>
-      <c r="B49" s="2" t="s">
-        <v>290</v>
-      </c>
-      <c r="C49" s="2" t="s">
-        <v>180</v>
       </c>
       <c r="D49" s="1">
         <v>4</v>
@@ -2414,18 +2414,18 @@
         <v>144</v>
       </c>
       <c r="G49" s="2" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A50" s="2" t="s">
         <v>181</v>
       </c>
-    </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A50" s="2" t="s">
+      <c r="B50" s="2" t="s">
+        <v>290</v>
+      </c>
+      <c r="C50" s="2" t="s">
         <v>182</v>
-      </c>
-      <c r="B50" s="2" t="s">
-        <v>291</v>
-      </c>
-      <c r="C50" s="2" t="s">
-        <v>183</v>
       </c>
       <c r="D50" s="1">
         <v>4</v>
@@ -2437,18 +2437,18 @@
         <v>144</v>
       </c>
       <c r="G50" s="2" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A51" s="2" t="s">
         <v>184</v>
       </c>
-    </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A51" s="2" t="s">
+      <c r="B51" s="2" t="s">
+        <v>291</v>
+      </c>
+      <c r="C51" s="2" t="s">
         <v>185</v>
-      </c>
-      <c r="B51" s="2" t="s">
-        <v>292</v>
-      </c>
-      <c r="C51" s="2" t="s">
-        <v>186</v>
       </c>
       <c r="D51" s="1">
         <v>4</v>
@@ -2460,18 +2460,18 @@
         <v>144</v>
       </c>
       <c r="G51" s="2" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A52" s="2" t="s">
         <v>187</v>
       </c>
-    </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A52" s="2" t="s">
+      <c r="B52" s="2" t="s">
+        <v>279</v>
+      </c>
+      <c r="C52" s="2" t="s">
         <v>188</v>
-      </c>
-      <c r="B52" s="2" t="s">
-        <v>280</v>
-      </c>
-      <c r="C52" s="2" t="s">
-        <v>189</v>
       </c>
       <c r="D52" s="1">
         <v>1</v>
@@ -2486,38 +2486,38 @@
         <v>151</v>
       </c>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A53" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="B53" s="2" t="s">
         <v>190</v>
       </c>
-      <c r="B53" s="2" t="s">
+      <c r="C53" s="2" t="s">
         <v>191</v>
       </c>
-      <c r="C53" s="2" t="s">
+      <c r="D53" s="1">
+        <v>1</v>
+      </c>
+      <c r="E53" s="2" t="s">
         <v>192</v>
       </c>
-      <c r="D53" s="1">
-        <v>1</v>
-      </c>
-      <c r="E53" s="2" t="s">
+      <c r="F53" s="2" t="s">
         <v>193</v>
       </c>
-      <c r="F53" s="2" t="s">
+      <c r="G53" s="2" t="s">
         <v>194</v>
       </c>
-      <c r="G53" s="2" t="s">
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A54" s="2" t="s">
         <v>195</v>
       </c>
-    </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A54" s="2" t="s">
+      <c r="B54" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="C54" s="2" t="s">
         <v>196</v>
-      </c>
-      <c r="B54" s="2" t="s">
-        <v>293</v>
-      </c>
-      <c r="C54" s="2" t="s">
-        <v>197</v>
       </c>
       <c r="D54" s="1">
         <v>2</v>
@@ -2529,352 +2529,352 @@
         <v>144</v>
       </c>
       <c r="G54" s="2" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A55" s="2" t="s">
         <v>198</v>
       </c>
-    </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A55" s="2" t="s">
+      <c r="B55" s="2" t="s">
         <v>199</v>
       </c>
-      <c r="B55" s="2" t="s">
+      <c r="C55" s="2" t="s">
         <v>200</v>
-      </c>
-      <c r="C55" s="2" t="s">
-        <v>201</v>
       </c>
       <c r="D55" s="1">
         <v>2</v>
       </c>
       <c r="E55" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="F55" s="2" t="s">
         <v>202</v>
       </c>
-      <c r="F55" s="2" t="s">
+      <c r="G55" s="2" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A56" s="2" t="s">
         <v>203</v>
       </c>
-      <c r="G55" s="2" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A56" s="2" t="s">
+      <c r="B56" s="2" t="s">
+        <v>293</v>
+      </c>
+      <c r="C56" s="2" t="s">
         <v>204</v>
-      </c>
-      <c r="B56" s="2" t="s">
-        <v>294</v>
-      </c>
-      <c r="C56" s="2" t="s">
-        <v>205</v>
       </c>
       <c r="D56" s="1">
         <v>2</v>
       </c>
       <c r="E56" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="F56" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="G56" s="2" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A57" s="2" t="s">
         <v>206</v>
       </c>
-      <c r="F56" s="2" t="s">
-        <v>203</v>
-      </c>
-      <c r="G56" s="2" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A57" s="2" t="s">
+      <c r="B57" s="2" t="s">
         <v>207</v>
       </c>
-      <c r="B57" s="2" t="s">
+      <c r="C57" s="2" t="s">
         <v>208</v>
       </c>
-      <c r="C57" s="2" t="s">
+      <c r="D57" s="1">
+        <v>1</v>
+      </c>
+      <c r="E57" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="F57" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="G57" s="2" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A58" s="2" t="s">
         <v>209</v>
       </c>
-      <c r="D57" s="1">
-        <v>1</v>
-      </c>
-      <c r="E57" s="2" t="s">
-        <v>207</v>
-      </c>
-      <c r="F57" s="2" t="s">
-        <v>203</v>
-      </c>
-      <c r="G57" s="2" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A58" s="2" t="s">
+      <c r="B58" s="2" t="s">
         <v>210</v>
       </c>
-      <c r="B58" s="2" t="s">
+      <c r="C58" s="2" t="s">
         <v>211</v>
       </c>
-      <c r="C58" s="2" t="s">
+      <c r="D58" s="1">
+        <v>1</v>
+      </c>
+      <c r="E58" s="2" t="s">
         <v>212</v>
       </c>
-      <c r="D58" s="1">
-        <v>1</v>
-      </c>
-      <c r="E58" s="2" t="s">
+      <c r="F58" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="G58" s="2" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A59" s="2" t="s">
         <v>213</v>
       </c>
-      <c r="F58" s="2" t="s">
-        <v>203</v>
-      </c>
-      <c r="G58" s="2" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A59" s="2" t="s">
+      <c r="B59" s="2" t="s">
         <v>214</v>
       </c>
-      <c r="B59" s="2" t="s">
+      <c r="C59" s="2" t="s">
         <v>215</v>
-      </c>
-      <c r="C59" s="2" t="s">
-        <v>216</v>
       </c>
       <c r="D59" s="1">
         <v>4</v>
       </c>
       <c r="E59" s="2" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="F59" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="G59" s="2" t="s">
         <v>217</v>
       </c>
-      <c r="G59" s="2" t="s">
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A60" s="2" t="s">
         <v>218</v>
       </c>
-    </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A60" s="2" t="s">
+      <c r="B60" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="B60" s="2" t="s">
+      <c r="C60" s="2" t="s">
         <v>220</v>
       </c>
-      <c r="C60" s="2" t="s">
+      <c r="D60" s="1">
+        <v>1</v>
+      </c>
+      <c r="E60" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="F60" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="G60" s="2" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A61" s="2" t="s">
         <v>221</v>
       </c>
-      <c r="D60" s="1">
-        <v>1</v>
-      </c>
-      <c r="E60" s="2" t="s">
-        <v>219</v>
-      </c>
-      <c r="F60" s="2" t="s">
-        <v>217</v>
-      </c>
-      <c r="G60" s="2" t="s">
-        <v>219</v>
-      </c>
-    </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A61" s="2" t="s">
+      <c r="B61" s="2" t="s">
         <v>222</v>
       </c>
-      <c r="B61" s="2" t="s">
+      <c r="C61" s="2" t="s">
         <v>223</v>
       </c>
-      <c r="C61" s="2" t="s">
+      <c r="D61" s="1">
+        <v>1</v>
+      </c>
+      <c r="E61" s="2" t="s">
         <v>224</v>
       </c>
-      <c r="D61" s="1">
-        <v>1</v>
-      </c>
-      <c r="E61" s="2" t="s">
+      <c r="F61" s="2" t="s">
         <v>225</v>
       </c>
-      <c r="F61" s="2" t="s">
+      <c r="G61" s="2" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A62" s="2" t="s">
         <v>226</v>
       </c>
-      <c r="G61" s="2" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A62" s="2" t="s">
+      <c r="B62" s="2" t="s">
         <v>227</v>
       </c>
-      <c r="B62" s="2" t="s">
+      <c r="C62" s="2" t="s">
         <v>228</v>
-      </c>
-      <c r="C62" s="2" t="s">
-        <v>229</v>
       </c>
       <c r="D62" s="1">
         <v>4</v>
       </c>
       <c r="E62" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="F62" s="2" t="s">
         <v>230</v>
       </c>
-      <c r="F62" s="2" t="s">
+      <c r="G62" s="2" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A63" s="2" t="s">
         <v>231</v>
       </c>
-      <c r="G62" s="2" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A63" s="2" t="s">
+      <c r="B63" s="2" t="s">
+        <v>294</v>
+      </c>
+      <c r="C63" s="2" t="s">
         <v>232</v>
       </c>
-      <c r="B63" s="2" t="s">
+      <c r="D63" s="1">
+        <v>1</v>
+      </c>
+      <c r="E63" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="F63" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="G63" s="2" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A64" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="B64" s="2" t="s">
         <v>295</v>
       </c>
-      <c r="C63" s="2" t="s">
-        <v>233</v>
-      </c>
-      <c r="D63" s="1">
-        <v>1</v>
-      </c>
-      <c r="E63" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="F63" s="2" t="s">
-        <v>235</v>
-      </c>
-      <c r="G63" s="2" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A64" s="2" t="s">
+      <c r="C64" s="2" t="s">
         <v>236</v>
-      </c>
-      <c r="B64" s="2" t="s">
-        <v>296</v>
-      </c>
-      <c r="C64" s="2" t="s">
-        <v>237</v>
       </c>
       <c r="D64" s="1">
         <v>4</v>
       </c>
       <c r="E64" s="2" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="F64" s="2" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="G64" s="2" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A65" s="2" t="s">
         <v>238</v>
       </c>
-    </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A65" s="2" t="s">
+      <c r="B65" s="2" t="s">
+        <v>296</v>
+      </c>
+      <c r="C65" s="2" t="s">
         <v>239</v>
-      </c>
-      <c r="B65" s="2" t="s">
-        <v>297</v>
-      </c>
-      <c r="C65" s="2" t="s">
-        <v>240</v>
       </c>
       <c r="D65" s="1">
         <v>2</v>
       </c>
       <c r="E65" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="F65" s="2" t="s">
         <v>241</v>
       </c>
-      <c r="F65" s="2" t="s">
+      <c r="G65" s="2" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A66" s="2" t="s">
         <v>242</v>
       </c>
-      <c r="G65" s="2" t="s">
-        <v>239</v>
-      </c>
-    </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A66" s="2" t="s">
+      <c r="B66" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="B66" s="2" t="s">
+      <c r="C66" s="2" t="s">
         <v>244</v>
       </c>
-      <c r="C66" s="2" t="s">
+      <c r="D66" s="1">
+        <v>1</v>
+      </c>
+      <c r="E66" s="2" t="s">
         <v>245</v>
       </c>
-      <c r="D66" s="1">
-        <v>1</v>
-      </c>
-      <c r="E66" s="2" t="s">
+      <c r="F66" s="2" t="s">
         <v>246</v>
       </c>
-      <c r="F66" s="2" t="s">
+      <c r="G66" s="2" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="67" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A67" s="2" t="s">
         <v>247</v>
       </c>
-      <c r="G66" s="2" t="s">
-        <v>243</v>
-      </c>
-    </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A67" s="2" t="s">
+      <c r="B67" s="2" t="s">
         <v>248</v>
       </c>
-      <c r="B67" s="2" t="s">
+      <c r="C67" s="2" t="s">
         <v>249</v>
       </c>
-      <c r="C67" s="2" t="s">
+      <c r="D67" s="1">
+        <v>1</v>
+      </c>
+      <c r="E67" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="F67" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="G67" s="2" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A68" s="2" t="s">
         <v>250</v>
       </c>
-      <c r="D67" s="1">
-        <v>1</v>
-      </c>
-      <c r="E67" s="2" t="s">
-        <v>248</v>
-      </c>
-      <c r="F67" s="2" t="s">
-        <v>203</v>
-      </c>
-      <c r="G67" s="2" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A68" s="2" t="s">
+      <c r="B68" s="2" t="s">
         <v>251</v>
       </c>
-      <c r="B68" s="2" t="s">
+      <c r="C68" s="2" t="s">
         <v>252</v>
       </c>
-      <c r="C68" s="2" t="s">
+      <c r="D68" s="1">
+        <v>1</v>
+      </c>
+      <c r="E68" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="F68" s="2" t="s">
         <v>253</v>
       </c>
-      <c r="D68" s="1">
-        <v>1</v>
-      </c>
-      <c r="E68" s="2" t="s">
-        <v>251</v>
-      </c>
-      <c r="F68" s="2" t="s">
+      <c r="G68" s="2" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A69" s="2" t="s">
         <v>254</v>
       </c>
-      <c r="G68" s="2" t="s">
-        <v>251</v>
-      </c>
-    </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A69" s="2" t="s">
+      <c r="B69" s="2" t="s">
         <v>255</v>
       </c>
-      <c r="B69" s="2" t="s">
+      <c r="C69" s="2" t="s">
         <v>256</v>
       </c>
-      <c r="C69" s="2" t="s">
+      <c r="D69" s="1">
+        <v>1</v>
+      </c>
+      <c r="E69" s="2" t="s">
         <v>257</v>
       </c>
-      <c r="D69" s="1">
-        <v>1</v>
-      </c>
-      <c r="E69" s="2" t="s">
+      <c r="F69" s="2" t="s">
         <v>258</v>
       </c>
-      <c r="F69" s="2" t="s">
+      <c r="G69" s="2" t="s">
         <v>259</v>
-      </c>
-      <c r="G69" s="2" t="s">
-        <v>260</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
EXP_V121 | 13/04/25 | 15:38
</commit_message>
<xml_diff>
--- a/03_BOM/EXP_V121_BOM.xlsx
+++ b/03_BOM/EXP_V121_BOM.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\LAB\NANORACK_V2_EXP_1.1.1_HW\03_BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2F194ED-F795-427F-8A37-495763D98C9D}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{514999C3-BCBF-40E5-930D-FD5EB13DD3D8}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{CB84624A-87DC-4816-B95B-F0221E4A3080}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{4D4FAE15-85C0-4811-B0C6-0F62DF96332D}"/>
   </bookViews>
   <sheets>
-    <sheet name="EXP_V121_BOM1" sheetId="1" r:id="rId1"/>
+    <sheet name="EXP_HW_V3" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Titles" localSheetId="0">EXP_V121_BOM1!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">EXP_HW_V3!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="405" uniqueCount="298">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="411" uniqueCount="300">
   <si>
     <t>Name</t>
   </si>
@@ -489,7 +489,7 @@
     <t>22R</t>
   </si>
   <si>
-    <t>R4, R8, R15, R25, R26, R45, R47, R48, R49, R50, R51, R52, R53, R54, R55, R66, R67, R68, R69, R72, R73, R74, R75, R78, R79, R80, R81, R84, R85, R86, R87, R94, R95, R96, R97, R105, R106, R107, R113, R114, R115, R116, R117, R118, R119, R120, R121, R122, R123, R124, R125, R126, R127, R128, R129, R130, R131, R132, R133, R134, R141, R142, R143, R144, R154, R157, R159, R161, R162, R167</t>
+    <t>R4, R8, R15, R25, R26, R45, R47, R48, R49, R50, R51, R52, R53, R54, R55, R66, R67, R68, R69, R72, R73, R74, R75, R78, R79, R80, R81, R84, R85, R86, R87, R94, R95, R96, R97, R105, R106, R107, R113, R114, R115, R116, R117, R118, R119, R120, R121, R122, R123, R124, R125, R126, R127, R128, R129, R130, R131, R132, R133, R134, R141, R142, R143, R144, R154, R157, R159, R167</t>
   </si>
   <si>
     <t>ERJ-3EKF22R0V</t>
@@ -498,6 +498,9 @@
     <t>4.7k</t>
   </si>
   <si>
+    <t>R5, R40, R41, R42, R43, R44, R90, R91, R92, R93, R99, R100, R139, R140, R153, R155, R163, R164, R165, R166, R168</t>
+  </si>
+  <si>
     <t>ERJ-3EKF4701V</t>
   </si>
   <si>
@@ -624,6 +627,12 @@
     <t>ERJ-3EKF1652V</t>
   </si>
   <si>
+    <t>22R/DNP</t>
+  </si>
+  <si>
+    <t>R161, R162</t>
+  </si>
+  <si>
     <t>TVS2200DRVR</t>
   </si>
   <si>
@@ -919,9 +928,6 @@
   </si>
   <si>
     <t>IC REDRIVER I2C HOTSWAP 8TSSOP</t>
-  </si>
-  <si>
-    <t>R5, R40, R41, R42, R43, R44, R90, R91, R92, R93, R99, R100, R139, R140, R153, R155, R163, R164, R165, R166, R168</t>
   </si>
 </sst>
 </file>
@@ -1297,17 +1303,17 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{81B74A45-8FA9-438A-BE1B-5C4E575BDB90}">
-  <dimension ref="A1:G69"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E3B2A7F-E6EE-4777-848D-203136C36565}">
+  <dimension ref="A1:G70"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.7265625" customWidth="1"/>
-    <col min="2" max="2" width="72.453125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="32" customWidth="1"/>
-    <col min="4" max="4" width="10.81640625" customWidth="1"/>
-    <col min="5" max="5" width="36.26953125" customWidth="1"/>
-    <col min="6" max="6" width="16.453125" customWidth="1"/>
-    <col min="7" max="7" width="31.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.81640625" customWidth="1"/>
+    <col min="2" max="2" width="62.6328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="30.6328125" customWidth="1"/>
+    <col min="4" max="4" width="10.36328125" customWidth="1"/>
+    <col min="5" max="5" width="45.7265625" customWidth="1"/>
+    <col min="6" max="6" width="15.6328125" customWidth="1"/>
+    <col min="7" max="7" width="25.81640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.35">
@@ -1361,7 +1367,7 @@
         <v>13</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>14</v>
@@ -1384,7 +1390,7 @@
         <v>18</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>20</v>
@@ -1407,7 +1413,7 @@
         <v>24</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>25</v>
@@ -1430,7 +1436,7 @@
         <v>27</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>28</v>
@@ -1453,7 +1459,7 @@
         <v>30</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>31</v>
@@ -1476,7 +1482,7 @@
         <v>32</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>33</v>
@@ -1499,7 +1505,7 @@
         <v>35</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>36</v>
@@ -1522,7 +1528,7 @@
         <v>38</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>39</v>
@@ -1545,7 +1551,7 @@
         <v>41</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>42</v>
@@ -1568,7 +1574,7 @@
         <v>45</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>46</v>
@@ -1591,7 +1597,7 @@
         <v>48</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>49</v>
@@ -1660,7 +1666,7 @@
         <v>61</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>62</v>
@@ -1683,7 +1689,7 @@
         <v>66</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="C17" s="2" t="s">
         <v>67</v>
@@ -1706,7 +1712,7 @@
         <v>69</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
       <c r="C18" s="2" t="s">
         <v>70</v>
@@ -1729,7 +1735,7 @@
         <v>72</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
       <c r="C19" s="2" t="s">
         <v>73</v>
@@ -1794,7 +1800,7 @@
         <v>82</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="C22" s="2" t="s">
         <v>83</v>
@@ -2031,7 +2037,7 @@
         <v>123</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="C33" s="2" t="s">
         <v>124</v>
@@ -2077,7 +2083,7 @@
         <v>131</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="C35" s="2" t="s">
         <v>132</v>
@@ -2123,7 +2129,7 @@
         <v>141</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
       <c r="C37" s="2" t="s">
         <v>142</v>
@@ -2146,7 +2152,7 @@
         <v>146</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="C38" s="2" t="s">
         <v>147</v>
@@ -2169,7 +2175,7 @@
         <v>149</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="C39" s="2" t="s">
         <v>150</v>
@@ -2192,13 +2198,13 @@
         <v>152</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="C40" s="2" t="s">
         <v>153</v>
       </c>
       <c r="D40" s="1">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="E40" s="2" t="s">
         <v>143</v>
@@ -2215,10 +2221,10 @@
         <v>155</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>297</v>
+        <v>156</v>
       </c>
       <c r="D41" s="1">
         <v>21</v>
@@ -2230,18 +2236,18 @@
         <v>144</v>
       </c>
       <c r="G41" s="2" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A42" s="2" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D42" s="1">
         <v>1</v>
@@ -2253,18 +2259,18 @@
         <v>144</v>
       </c>
       <c r="G42" s="2" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A43" s="2" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D43" s="1">
         <v>9</v>
@@ -2276,18 +2282,18 @@
         <v>144</v>
       </c>
       <c r="G43" s="2" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A44" s="2" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D44" s="1">
         <v>5</v>
@@ -2299,18 +2305,18 @@
         <v>144</v>
       </c>
       <c r="G44" s="2" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A45" s="2" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D45" s="1">
         <v>1</v>
@@ -2322,18 +2328,18 @@
         <v>144</v>
       </c>
       <c r="G45" s="2" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A46" s="2" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="D46" s="1">
         <v>6</v>
@@ -2345,18 +2351,18 @@
         <v>144</v>
       </c>
       <c r="G46" s="2" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A47" s="2" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D47" s="1">
         <v>1</v>
@@ -2368,18 +2374,18 @@
         <v>144</v>
       </c>
       <c r="G47" s="2" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A48" s="2" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="D48" s="1">
         <v>4</v>
@@ -2391,18 +2397,18 @@
         <v>144</v>
       </c>
       <c r="G48" s="2" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A49" s="2" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="D49" s="1">
         <v>4</v>
@@ -2414,18 +2420,18 @@
         <v>144</v>
       </c>
       <c r="G49" s="2" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A50" s="2" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D50" s="1">
         <v>4</v>
@@ -2437,18 +2443,18 @@
         <v>144</v>
       </c>
       <c r="G50" s="2" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A51" s="2" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="D51" s="1">
         <v>4</v>
@@ -2460,18 +2466,18 @@
         <v>144</v>
       </c>
       <c r="G51" s="2" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A52" s="2" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D52" s="1">
         <v>1</v>
@@ -2488,36 +2494,36 @@
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A53" s="2" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D53" s="1">
         <v>1</v>
       </c>
       <c r="E53" s="2" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="F53" s="2" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="G53" s="2" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A54" s="2" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="D54" s="1">
         <v>2</v>
@@ -2529,15 +2535,15 @@
         <v>144</v>
       </c>
       <c r="G54" s="2" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A55" s="2" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>199</v>
+        <v>283</v>
       </c>
       <c r="C55" s="2" t="s">
         <v>200</v>
@@ -2546,36 +2552,36 @@
         <v>2</v>
       </c>
       <c r="E55" s="2" t="s">
-        <v>201</v>
+        <v>143</v>
       </c>
       <c r="F55" s="2" t="s">
-        <v>202</v>
+        <v>144</v>
       </c>
       <c r="G55" s="2" t="s">
-        <v>198</v>
+        <v>154</v>
       </c>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A56" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="B56" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="C56" s="2" t="s">
         <v>203</v>
-      </c>
-      <c r="B56" s="2" t="s">
-        <v>293</v>
-      </c>
-      <c r="C56" s="2" t="s">
-        <v>204</v>
       </c>
       <c r="D56" s="1">
         <v>2</v>
       </c>
       <c r="E56" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="F56" s="2" t="s">
         <v>205</v>
       </c>
-      <c r="F56" s="2" t="s">
-        <v>202</v>
-      </c>
       <c r="G56" s="2" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.35">
@@ -2583,19 +2589,19 @@
         <v>206</v>
       </c>
       <c r="B57" s="2" t="s">
+        <v>296</v>
+      </c>
+      <c r="C57" s="2" t="s">
         <v>207</v>
       </c>
-      <c r="C57" s="2" t="s">
+      <c r="D57" s="1">
+        <v>2</v>
+      </c>
+      <c r="E57" s="2" t="s">
         <v>208</v>
       </c>
-      <c r="D57" s="1">
-        <v>1</v>
-      </c>
-      <c r="E57" s="2" t="s">
-        <v>206</v>
-      </c>
       <c r="F57" s="2" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="G57" s="2" t="s">
         <v>206</v>
@@ -2615,10 +2621,10 @@
         <v>1</v>
       </c>
       <c r="E58" s="2" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="F58" s="2" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="G58" s="2" t="s">
         <v>209</v>
@@ -2626,48 +2632,48 @@
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A59" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="B59" s="2" t="s">
         <v>213</v>
       </c>
-      <c r="B59" s="2" t="s">
+      <c r="C59" s="2" t="s">
         <v>214</v>
       </c>
-      <c r="C59" s="2" t="s">
+      <c r="D59" s="1">
+        <v>1</v>
+      </c>
+      <c r="E59" s="2" t="s">
         <v>215</v>
       </c>
-      <c r="D59" s="1">
-        <v>4</v>
-      </c>
-      <c r="E59" s="2" t="s">
-        <v>213</v>
-      </c>
       <c r="F59" s="2" t="s">
-        <v>216</v>
+        <v>205</v>
       </c>
       <c r="G59" s="2" t="s">
-        <v>217</v>
+        <v>212</v>
       </c>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A60" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="B60" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="C60" s="2" t="s">
         <v>218</v>
       </c>
-      <c r="B60" s="2" t="s">
+      <c r="D60" s="1">
+        <v>4</v>
+      </c>
+      <c r="E60" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="F60" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="C60" s="2" t="s">
+      <c r="G60" s="2" t="s">
         <v>220</v>
-      </c>
-      <c r="D60" s="1">
-        <v>1</v>
-      </c>
-      <c r="E60" s="2" t="s">
-        <v>218</v>
-      </c>
-      <c r="F60" s="2" t="s">
-        <v>216</v>
-      </c>
-      <c r="G60" s="2" t="s">
-        <v>218</v>
       </c>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.35">
@@ -2684,10 +2690,10 @@
         <v>1</v>
       </c>
       <c r="E61" s="2" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="F61" s="2" t="s">
-        <v>225</v>
+        <v>219</v>
       </c>
       <c r="G61" s="2" t="s">
         <v>221</v>
@@ -2695,71 +2701,71 @@
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A62" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="B62" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="C62" s="2" t="s">
         <v>226</v>
       </c>
-      <c r="B62" s="2" t="s">
+      <c r="D62" s="1">
+        <v>1</v>
+      </c>
+      <c r="E62" s="2" t="s">
         <v>227</v>
       </c>
-      <c r="C62" s="2" t="s">
+      <c r="F62" s="2" t="s">
         <v>228</v>
       </c>
-      <c r="D62" s="1">
-        <v>4</v>
-      </c>
-      <c r="E62" s="2" t="s">
-        <v>229</v>
-      </c>
-      <c r="F62" s="2" t="s">
-        <v>230</v>
-      </c>
       <c r="G62" s="2" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A63" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="B63" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="C63" s="2" t="s">
         <v>231</v>
       </c>
-      <c r="B63" s="2" t="s">
-        <v>294</v>
-      </c>
-      <c r="C63" s="2" t="s">
+      <c r="D63" s="1">
+        <v>4</v>
+      </c>
+      <c r="E63" s="2" t="s">
         <v>232</v>
       </c>
-      <c r="D63" s="1">
-        <v>1</v>
-      </c>
-      <c r="E63" s="2" t="s">
+      <c r="F63" s="2" t="s">
         <v>233</v>
       </c>
-      <c r="F63" s="2" t="s">
-        <v>234</v>
-      </c>
       <c r="G63" s="2" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A64" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="B64" s="2" t="s">
+        <v>297</v>
+      </c>
+      <c r="C64" s="2" t="s">
         <v>235</v>
       </c>
-      <c r="B64" s="2" t="s">
-        <v>295</v>
-      </c>
-      <c r="C64" s="2" t="s">
+      <c r="D64" s="1">
+        <v>1</v>
+      </c>
+      <c r="E64" s="2" t="s">
         <v>236</v>
       </c>
-      <c r="D64" s="1">
-        <v>4</v>
-      </c>
-      <c r="E64" s="2" t="s">
-        <v>229</v>
-      </c>
       <c r="F64" s="2" t="s">
-        <v>202</v>
+        <v>237</v>
       </c>
       <c r="G64" s="2" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.35">
@@ -2767,68 +2773,68 @@
         <v>238</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="C65" s="2" t="s">
         <v>239</v>
       </c>
       <c r="D65" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E65" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="F65" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="G65" s="2" t="s">
         <v>240</v>
-      </c>
-      <c r="F65" s="2" t="s">
-        <v>241</v>
-      </c>
-      <c r="G65" s="2" t="s">
-        <v>238</v>
       </c>
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A66" s="2" t="s">
+        <v>241</v>
+      </c>
+      <c r="B66" s="2" t="s">
+        <v>299</v>
+      </c>
+      <c r="C66" s="2" t="s">
         <v>242</v>
       </c>
-      <c r="B66" s="2" t="s">
+      <c r="D66" s="1">
+        <v>2</v>
+      </c>
+      <c r="E66" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="C66" s="2" t="s">
+      <c r="F66" s="2" t="s">
         <v>244</v>
       </c>
-      <c r="D66" s="1">
-        <v>1</v>
-      </c>
-      <c r="E66" s="2" t="s">
-        <v>245</v>
-      </c>
-      <c r="F66" s="2" t="s">
-        <v>246</v>
-      </c>
       <c r="G66" s="2" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A67" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="B67" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="C67" s="2" t="s">
         <v>247</v>
       </c>
-      <c r="B67" s="2" t="s">
+      <c r="D67" s="1">
+        <v>1</v>
+      </c>
+      <c r="E67" s="2" t="s">
         <v>248</v>
       </c>
-      <c r="C67" s="2" t="s">
+      <c r="F67" s="2" t="s">
         <v>249</v>
       </c>
-      <c r="D67" s="1">
-        <v>1</v>
-      </c>
-      <c r="E67" s="2" t="s">
-        <v>247</v>
-      </c>
-      <c r="F67" s="2" t="s">
-        <v>202</v>
-      </c>
       <c r="G67" s="2" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.35">
@@ -2848,7 +2854,7 @@
         <v>250</v>
       </c>
       <c r="F68" s="2" t="s">
-        <v>253</v>
+        <v>205</v>
       </c>
       <c r="G68" s="2" t="s">
         <v>250</v>
@@ -2856,25 +2862,48 @@
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A69" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="B69" s="2" t="s">
         <v>254</v>
       </c>
-      <c r="B69" s="2" t="s">
+      <c r="C69" s="2" t="s">
         <v>255</v>
       </c>
-      <c r="C69" s="2" t="s">
+      <c r="D69" s="1">
+        <v>1</v>
+      </c>
+      <c r="E69" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="F69" s="2" t="s">
         <v>256</v>
       </c>
-      <c r="D69" s="1">
-        <v>1</v>
-      </c>
-      <c r="E69" s="2" t="s">
+      <c r="G69" s="2" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A70" s="2" t="s">
         <v>257</v>
       </c>
-      <c r="F69" s="2" t="s">
+      <c r="B70" s="2" t="s">
         <v>258</v>
       </c>
-      <c r="G69" s="2" t="s">
+      <c r="C70" s="2" t="s">
         <v>259</v>
+      </c>
+      <c r="D70" s="1">
+        <v>1</v>
+      </c>
+      <c r="E70" s="2" t="s">
+        <v>260</v>
+      </c>
+      <c r="F70" s="2" t="s">
+        <v>261</v>
+      </c>
+      <c r="G70" s="2" t="s">
+        <v>262</v>
       </c>
     </row>
   </sheetData>

</xml_diff>